<commit_message>
fix(templates): update EMAX PI template and mapping
根据实际模板文件更新：
- Column C = Item Number (SAP) / Item Line#
- Column G = USD Amount（新列，之前没有）
- 新增 ex_factory_date / document_date header 引用
- Total 从 G24 改为 F24
</commit_message>
<xml_diff>
--- a/templates/emax/pi.xlsx
+++ b/templates/emax/pi.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6550"/>
+    <workbookView windowWidth="29400" windowHeight="14100"/>
   </bookViews>
   <sheets>
     <sheet name="PF Standard Invoice format" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>E MAX SPORT PTE. LTD.</t>
   </si>
@@ -45,56 +45,18 @@
     <t>PI Number:</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>RO new PO template A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>列</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>"Purchasing Document"</t>
-    </r>
-  </si>
-  <si>
     <t>Document Date:</t>
   </si>
   <si>
-    <t>生成日期</t>
-  </si>
-  <si>
     <t>Payment Terms:</t>
   </si>
   <si>
     <t>Net 90 days</t>
   </si>
   <si>
-    <t>固定值</t>
-  </si>
-  <si>
     <t>Shipment Ex-factory Date:</t>
   </si>
   <si>
-    <t>手动更新</t>
-  </si>
-  <si>
     <t>Bill To:</t>
   </si>
   <si>
@@ -104,24 +66,12 @@
     <t>Ship to:</t>
   </si>
   <si>
-    <t>Rather Outdoors Corporation</t>
-  </si>
-  <si>
-    <t>套装ship to地址不同</t>
-  </si>
-  <si>
     <t>Columbia, South Carolina 29210</t>
   </si>
   <si>
-    <t>6505 Tower Lane</t>
-  </si>
-  <si>
     <t>United States</t>
   </si>
   <si>
-    <t>Claremore, OK 74019-4429</t>
-  </si>
-  <si>
     <t>Port of Loading:</t>
   </si>
   <si>
@@ -146,208 +96,6 @@
     <t>#08-32,PREMIER @ KAKI BUKIT, SINGAPORE 415875</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>RO new PO template I</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>列</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>"Material"</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>RO new PO template J</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>列</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>"Model",</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> ZEBCO</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>和</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>LEW'S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>是否取同一列</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>data base M</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>或</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>O</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>列</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>RO new PO template N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>列</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> “Order Quantity”</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>E</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>列</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>*F</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>列</t>
-    </r>
-  </si>
-  <si>
-    <t>EMAX/GS to GS PTE PI</t>
-  </si>
-  <si>
     <t>Country of The Origin</t>
   </si>
   <si>
@@ -372,46 +120,10 @@
     <t>EX-FACTORY DATE</t>
   </si>
   <si>
-    <t>4500030844</t>
-  </si>
-  <si>
-    <t>21-44900</t>
-  </si>
-  <si>
-    <t>ACA Merit 3000 7' 1PC ML 8-15 SP Combo</t>
-  </si>
-  <si>
-    <t>21-44625</t>
-  </si>
-  <si>
-    <t>Merit 5000 7' 1PC M 12-20 Spin Combo</t>
-  </si>
-  <si>
-    <t>21-44628</t>
-  </si>
-  <si>
-    <t>Merit 5000 8' 2PC MH 12-25 Spin Combo</t>
-  </si>
-  <si>
-    <t>21-44630</t>
-  </si>
-  <si>
-    <t>Merit 6000 7' 1PC MH 12-25 Spin Combo</t>
-  </si>
-  <si>
-    <t>21-44633</t>
-  </si>
-  <si>
-    <t>Merit 6000 9' 2PC MH 15-30 Spin Combo</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
     <t>Signature:</t>
-  </si>
-  <si>
-    <t>Joyce</t>
   </si>
   <si>
     <t>Date:</t>
@@ -2347,12 +2059,12 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I28"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.6"/>
   <cols>
     <col min="1" max="1" width="17.75" style="5" customWidth="1"/>
     <col min="2" max="2" width="13" style="5" customWidth="1"/>
     <col min="3" max="3" width="11" style="5" customWidth="1"/>
-    <col min="4" max="4" width="31.8333333333333" style="5" customWidth="1"/>
+    <col min="4" max="4" width="31.8303571428571" style="5" customWidth="1"/>
     <col min="5" max="5" width="13" style="5" customWidth="1"/>
     <col min="6" max="6" width="12.75" style="5" customWidth="1"/>
     <col min="7" max="7" width="13.125" style="5" customWidth="1"/>
@@ -2416,44 +2128,30 @@
       <c r="A6" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="18">
-        <v>4500030844</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>4</v>
-      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="19"/>
       <c r="E6" s="12"/>
       <c r="F6" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="G6" s="20">
-        <v>46052</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>6</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G6" s="20"/>
+      <c r="H6" s="21"/>
       <c r="I6" s="22"/>
     </row>
     <row r="7" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
       <c r="A7" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>9</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="C7" s="24"/>
       <c r="E7" s="12"/>
       <c r="F7" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" s="25">
-        <v>46162</v>
-      </c>
-      <c r="H7" s="26" t="s">
-        <v>11</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="G7" s="25"/>
+      <c r="H7" s="26"/>
       <c r="I7" s="22"/>
     </row>
     <row r="8" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
@@ -2466,64 +2164,46 @@
     </row>
     <row r="9" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
       <c r="A9" s="27" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C9" s="31"/>
-      <c r="D9" s="24" t="s">
-        <v>9</v>
-      </c>
+      <c r="D9" s="24"/>
       <c r="E9" s="32"/>
       <c r="F9" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="30" t="s">
-        <v>15</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="G9" s="30"/>
       <c r="H9" s="30"/>
-      <c r="I9" s="34" t="s">
-        <v>16</v>
-      </c>
+      <c r="I9" s="34"/>
     </row>
     <row r="10" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
       <c r="A10" s="35"/>
       <c r="B10" s="36" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C10" s="37"/>
-      <c r="D10" s="24" t="s">
-        <v>9</v>
-      </c>
+      <c r="D10" s="24"/>
       <c r="E10" s="32"/>
       <c r="F10" s="15"/>
-      <c r="G10" s="36" t="s">
-        <v>18</v>
-      </c>
+      <c r="G10" s="36"/>
       <c r="H10" s="36"/>
-      <c r="I10" s="34" t="s">
-        <v>16</v>
-      </c>
+      <c r="I10" s="34"/>
     </row>
     <row r="11" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
       <c r="A11" s="27"/>
       <c r="B11" s="36" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C11" s="37"/>
-      <c r="D11" s="24" t="s">
-        <v>9</v>
-      </c>
+      <c r="D11" s="24"/>
       <c r="E11" s="32"/>
       <c r="F11" s="38"/>
-      <c r="G11" s="36" t="s">
-        <v>20</v>
-      </c>
+      <c r="G11" s="36"/>
       <c r="H11" s="36"/>
-      <c r="I11" s="34" t="s">
-        <v>16</v>
-      </c>
+      <c r="I11" s="34"/>
     </row>
     <row r="12" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
       <c r="E12" s="32"/>
@@ -2534,49 +2214,41 @@
     </row>
     <row r="13" s="3" customFormat="1" ht="18.95" customHeight="1" spans="1:9">
       <c r="A13" s="12" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B13" s="41" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="24" t="s">
-        <v>9</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C13" s="24"/>
       <c r="D13" s="41"/>
       <c r="E13" s="32"/>
       <c r="F13" s="15" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="G13" s="42" t="s">
         <v>0</v>
       </c>
       <c r="H13" s="42"/>
-      <c r="I13" s="24" t="s">
-        <v>9</v>
-      </c>
+      <c r="I13" s="24"/>
     </row>
     <row r="14" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
       <c r="A14" s="12" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B14" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="24" t="s">
-        <v>9</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C14" s="24"/>
       <c r="D14" s="44"/>
       <c r="E14" s="32"/>
       <c r="F14" s="15" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G14" s="45" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H14" s="45"/>
-      <c r="I14" s="24" t="s">
-        <v>9</v>
-      </c>
+      <c r="I14" s="24"/>
     </row>
     <row r="15" s="3" customFormat="1" ht="24" customHeight="1" spans="1:9">
       <c r="A15" s="27"/>
@@ -2586,196 +2258,95 @@
       <c r="E15" s="32"/>
       <c r="F15" s="38"/>
       <c r="G15" s="46" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H15" s="46"/>
-      <c r="I15" s="24" t="s">
-        <v>9</v>
-      </c>
+      <c r="I15" s="24"/>
     </row>
     <row r="16" ht="38" customHeight="1" spans="1:9">
-      <c r="B16" s="47" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" s="47" t="s">
-        <v>29</v>
-      </c>
-      <c r="D16" s="47" t="s">
-        <v>30</v>
-      </c>
-      <c r="E16" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="F16" s="47" t="s">
-        <v>32</v>
-      </c>
-      <c r="G16" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="H16" s="47" t="s">
-        <v>34</v>
-      </c>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="47"/>
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:9">
       <c r="A17" s="48" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="B17" s="48" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="C17" s="49" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="D17" s="50" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="E17" s="51" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="F17" s="49" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="G17" s="52" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="H17" s="53" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="1:9">
-      <c r="A18" s="54" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="54" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="55" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="56" t="s">
-        <v>45</v>
-      </c>
-      <c r="E18" s="57">
-        <v>26.82</v>
-      </c>
-      <c r="F18" s="58">
-        <v>504</v>
-      </c>
-      <c r="G18" s="57">
-        <f>F18*E18</f>
-        <v>13517.28</v>
-      </c>
-      <c r="H18" s="59">
-        <v>46162</v>
-      </c>
+      <c r="A18" s="54"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="55"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="59"/>
     </row>
     <row r="19" ht="24" customHeight="1" spans="1:9">
-      <c r="A19" s="54" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="54" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" s="49" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="50" t="s">
-        <v>47</v>
-      </c>
-      <c r="E19" s="60">
-        <v>31.82</v>
-      </c>
-      <c r="F19" s="61">
-        <v>520</v>
-      </c>
-      <c r="G19" s="57">
-        <f>F19*E19</f>
-        <v>16546.4</v>
-      </c>
-      <c r="H19" s="59">
-        <v>46162</v>
-      </c>
+      <c r="A19" s="54"/>
+      <c r="B19" s="54"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="59"/>
     </row>
     <row r="20" ht="24" customHeight="1" spans="1:9">
-      <c r="A20" s="54" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="54" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="49" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="50" t="s">
-        <v>49</v>
-      </c>
-      <c r="E20" s="60">
-        <v>32.82</v>
-      </c>
-      <c r="F20" s="61">
-        <v>200</v>
-      </c>
-      <c r="G20" s="57">
-        <f>F20*E20</f>
-        <v>6564</v>
-      </c>
-      <c r="H20" s="59">
-        <v>46162</v>
-      </c>
+      <c r="A20" s="54"/>
+      <c r="B20" s="54"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="50"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="57"/>
+      <c r="H20" s="59"/>
     </row>
     <row r="21" ht="24" customHeight="1" spans="1:9">
-      <c r="A21" s="54" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="54" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="49" t="s">
-        <v>50</v>
-      </c>
-      <c r="D21" s="50" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" s="60">
-        <v>32.68</v>
-      </c>
-      <c r="F21" s="61">
-        <v>300</v>
-      </c>
-      <c r="G21" s="57">
-        <f>F21*E21</f>
-        <v>9804</v>
-      </c>
-      <c r="H21" s="59">
-        <v>46162</v>
-      </c>
+      <c r="A21" s="54"/>
+      <c r="B21" s="54"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="61"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="59"/>
     </row>
     <row r="22" ht="24" customHeight="1" spans="1:9">
-      <c r="A22" s="54" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="54" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="62" t="s">
-        <v>52</v>
-      </c>
-      <c r="D22" s="50" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="60">
-        <v>34.01</v>
-      </c>
-      <c r="F22" s="61">
-        <v>200</v>
-      </c>
-      <c r="G22" s="57">
-        <f>F22*E22</f>
-        <v>6802</v>
-      </c>
-      <c r="H22" s="59">
-        <v>46162</v>
-      </c>
+      <c r="A22" s="54"/>
+      <c r="B22" s="54"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="61"/>
+      <c r="G22" s="57"/>
+      <c r="H22" s="59"/>
     </row>
     <row r="23" ht="24" customHeight="1" spans="1:9">
       <c r="A23" s="63"/>
@@ -2795,12 +2366,9 @@
       <c r="D24" s="66"/>
       <c r="E24" s="67"/>
       <c r="F24" s="68" t="s">
-        <v>54</v>
-      </c>
-      <c r="G24" s="69">
-        <f>SUM(G18:G22)</f>
-        <v>53233.68</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G24" s="69"/>
       <c r="H24" s="70"/>
     </row>
     <row r="25" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
@@ -2809,28 +2377,20 @@
     <row r="26" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
       <c r="A26" s="72"/>
       <c r="F26" s="73" t="s">
-        <v>55</v>
-      </c>
-      <c r="G26" s="74" t="s">
-        <v>56</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="G26" s="74"/>
       <c r="H26" s="74"/>
-      <c r="I26" s="26" t="s">
-        <v>11</v>
-      </c>
+      <c r="I26" s="26"/>
     </row>
     <row r="27" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
       <c r="A27" s="72"/>
       <c r="F27" s="75" t="s">
-        <v>57</v>
-      </c>
-      <c r="G27" s="20">
-        <v>46052</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G27" s="20"/>
       <c r="H27" s="76"/>
-      <c r="I27" s="21" t="s">
-        <v>6</v>
-      </c>
+      <c r="I27" s="21"/>
     </row>
     <row r="28" s="4" customFormat="1" spans="1:9">
       <c r="I28" s="71"/>

</xml_diff>

<commit_message>
feat: complete Phase 3/4 - workbench MVP with launcher fix
- Add workbench service, workbook cache/snapshot/editor modules
- Add document preview, header/line/totals rules modules
- Update all 14 template mappings and xlsx files for Phase 3
- Add FastAPI workbench API endpoints with session management
- Add launcher startup error dialog when frontend/dist is missing
- Change launcher to console=False on Windows for clean UX
- Add icons.svg static route to app.py
- Add E2E tests for workbench API
- Add unified field mapping guide and design mockup docs
</commit_message>
<xml_diff>
--- a/templates/emax/pi.xlsx
+++ b/templates/emax/pi.xlsx
@@ -10,8 +10,7 @@
     <sheet name="PF Standard Invoice format" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PF Standard Invoice format'!$A$17:$H$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PF Standard Invoice format'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PF Standard Invoice format'!$A$1:$H$24</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>E MAX SPORT PTE. LTD.</t>
   </si>
@@ -51,31 +50,16 @@
     <t>Payment Terms:</t>
   </si>
   <si>
-    <t>Net 90 days</t>
-  </si>
-  <si>
     <t>Shipment Ex-factory Date:</t>
   </si>
   <si>
     <t>Bill To:</t>
   </si>
   <si>
-    <t>209 Stoneridge Drive</t>
-  </si>
-  <si>
     <t>Ship to:</t>
   </si>
   <si>
-    <t>Columbia, South Carolina 29210</t>
-  </si>
-  <si>
-    <t>United States</t>
-  </si>
-  <si>
     <t>Port of Loading:</t>
-  </si>
-  <si>
-    <t>China</t>
   </si>
   <si>
     <t>Actual Manufacturer Company Name</t>
@@ -84,16 +68,7 @@
     <t>Final Destination</t>
   </si>
   <si>
-    <t>USA</t>
-  </si>
-  <si>
     <t>Actual Manufacturer Company Address</t>
-  </si>
-  <si>
-    <t>8 KAKI BUKIT AVENUE 4</t>
-  </si>
-  <si>
-    <t>#08-32,PREMIER @ KAKI BUKIT, SINGAPORE 415875</t>
   </si>
   <si>
     <t>Country of The Origin</t>
@@ -173,13 +148,6 @@
     </font>
     <font>
       <b/>
-      <sz val="20"/>
-      <color theme="3" tint="0.399975585192419"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
       <sz val="8"/>
       <name val="Arial Black"/>
       <charset val="134"/>
@@ -193,8 +161,8 @@
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF00B0F0"/>
-      <name val="Arial"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
       <charset val="134"/>
     </font>
     <font>
@@ -204,6 +172,12 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <name val="Arial"/>
@@ -212,12 +186,12 @@
     <font>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
-      <name val="宋体"/>
+      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF00B0F0"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -809,7 +783,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -847,19 +821,6 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -1075,166 +1036,166 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="36" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="38" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="39" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="37" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="33" fillId="0" borderId="0"/>
@@ -1246,62 +1207,62 @@
     </xf>
     <xf numFmtId="176" fontId="35" fillId="0" borderId="0"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="32" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="32" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="32" fillId="39" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="36" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="40" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="41" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="39" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="32" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="39" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="42" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="43" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="41" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="39" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="35" fillId="0" borderId="0"/>
     <xf numFmtId="176" fontId="37" fillId="0" borderId="0"/>
     <xf numFmtId="176" fontId="38" fillId="0" borderId="0"/>
     <xf numFmtId="176" fontId="37" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="35" fillId="37" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="40" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="41" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="42" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="42" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="35" fillId="37" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="39" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="40" fillId="0" borderId="13">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="41" fillId="0" borderId="14">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="42" fillId="0" borderId="15">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="42" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="34" fillId="0" borderId="0">
@@ -1337,61 +1298,61 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="37" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="36" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="36" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="44" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="45" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="46" fillId="49" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="47" fillId="50" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="48" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="48" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="49" fillId="49" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="50" fillId="40" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="51" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="36" fillId="44" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="42" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="43" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="45" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="46" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="36" fillId="47" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="44" fillId="0" borderId="16">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="45" fillId="48" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="46" fillId="49" borderId="17">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="47" fillId="50" borderId="18">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="48" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="48" fillId="0" borderId="19">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="49" fillId="49" borderId="20">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="50" fillId="40" borderId="17">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="51" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="37" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="52" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="52" fillId="40" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="77">
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+  <cellXfs count="78">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1400,28 +1361,25 @@
     <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="86" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="0" xfId="86" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="86" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="0" xfId="86" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="0" xfId="86" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="86" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="0" xfId="86" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="176" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="55" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -1443,42 +1401,42 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="176" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="178" fontId="2" fillId="2" borderId="2" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="176" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="3" borderId="2" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="2" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="76" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1502,8 +1460,8 @@
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="176" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="176" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="88" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1531,6 +1489,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="176" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1545,7 +1506,16 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="2" borderId="0" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="77" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1566,23 +1536,14 @@
     <xf numFmtId="177" fontId="1" fillId="2" borderId="3" xfId="86" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="77" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="77" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="2" borderId="4" xfId="76" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="1" fillId="2" borderId="3" xfId="76" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="77" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="77" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="26" fontId="1" fillId="2" borderId="4" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="2" borderId="4" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="1" fillId="2" borderId="4" xfId="86" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="26" fontId="1" fillId="2" borderId="3" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1590,10 +1551,7 @@
     <xf numFmtId="180" fontId="1" fillId="2" borderId="3" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="2" borderId="3" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="77" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="1" fillId="2" borderId="3" xfId="86" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="181" fontId="1" fillId="2" borderId="0" xfId="86" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1602,10 +1560,10 @@
     <xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="11" fillId="2" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="2" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="10" fillId="2" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="2" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="2" fillId="2" borderId="0" xfId="98" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1617,22 +1575,29 @@
     <xf numFmtId="40" fontId="2" fillId="2" borderId="1" xfId="98" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="2" borderId="0" xfId="86" applyNumberFormat="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="177" fontId="6" fillId="2" borderId="0" xfId="76" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="2" borderId="0" xfId="86" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="2" borderId="0" xfId="75" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="86" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="86" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="2" borderId="0" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="2" borderId="0" xfId="86" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="2" xfId="86" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="2" xfId="86" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1755,12 +1720,6 @@
     <cellStyle name="中等" xfId="115"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="00FFFF99"/>
-      <color rgb="00FF0000"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2058,7 +2017,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.6"/>
   <cols>
     <col min="1" max="1" width="17.75" style="5" customWidth="1"/>
@@ -2070,341 +2029,275 @@
     <col min="7" max="7" width="13.125" style="5" customWidth="1"/>
     <col min="8" max="8" width="16.5" style="5" customWidth="1"/>
     <col min="9" max="9" width="11.375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="5"/>
+    <col min="10" max="16384" width="9" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="25.5" customHeight="1" spans="1:9">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="9"/>
+      <c r="I1" s="8"/>
     </row>
     <row r="2" s="1" customFormat="1" ht="21.95" customHeight="1" spans="1:9">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="9"/>
+      <c r="I2" s="8"/>
     </row>
     <row r="3" s="1" customFormat="1" ht="18.95" customHeight="1" spans="1:9">
-      <c r="I3" s="9"/>
+      <c r="I3" s="8"/>
     </row>
     <row r="4" s="1" customFormat="1" ht="27.95" customHeight="1" spans="1:9">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="9"/>
+      <c r="I4" s="8"/>
     </row>
     <row r="5" s="1" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A5" s="12"/>
-      <c r="B5" s="13"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="17"/>
-    </row>
-    <row r="6" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A6" s="12" t="s">
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="16"/>
+    </row>
+    <row r="6" s="2" customFormat="1" ht="37" customHeight="1" spans="1:9">
+      <c r="A6" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="15" t="s">
+      <c r="B6" s="17"/>
+      <c r="C6" s="18"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="20"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="22"/>
-    </row>
-    <row r="7" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A7" s="12" t="s">
+      <c r="G6" s="19"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="21"/>
+    </row>
+    <row r="7" s="2" customFormat="1" ht="33" customHeight="1" spans="1:9">
+      <c r="A7" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="22"/>
+      <c r="C7" s="23"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="15" t="s">
+      <c r="G7" s="24"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="21"/>
+    </row>
+    <row r="8" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="A8" s="26"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="28"/>
+    </row>
+    <row r="9" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="A9" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="22"/>
-    </row>
-    <row r="8" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A8" s="27"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="29"/>
-    </row>
-    <row r="9" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A9" s="27" t="s">
+      <c r="B9" s="29"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="33"/>
+    </row>
+    <row r="10" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="A10" s="34"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="35"/>
+    </row>
+    <row r="11" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="A11" s="26"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="35"/>
+    </row>
+    <row r="12" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="E12" s="31"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="39"/>
+    </row>
+    <row r="13" s="3" customFormat="1" ht="18.95" customHeight="1" spans="1:9">
+      <c r="A13" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="31"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="33" t="s">
+      <c r="B13" s="40"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="34"/>
-    </row>
-    <row r="10" s="2" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A10" s="35"/>
-      <c r="B10" s="36" t="s">
+      <c r="G13" s="41"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="23"/>
+    </row>
+    <row r="14" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="A14" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="34"/>
-    </row>
-    <row r="11" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A11" s="27"/>
-      <c r="B11" s="36" t="s">
+      <c r="B14" s="43"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="37"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="34"/>
-    </row>
-    <row r="12" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="E12" s="32"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="40"/>
-    </row>
-    <row r="13" s="3" customFormat="1" ht="18.95" customHeight="1" spans="1:9">
-      <c r="A13" s="12" t="s">
+      <c r="G14" s="45"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="23"/>
+    </row>
+    <row r="15" s="3" customFormat="1" ht="24" customHeight="1" spans="1:9">
+      <c r="A15" s="26"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="23"/>
+    </row>
+    <row r="16" ht="38" customHeight="1" spans="1:9">
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="48"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="50"/>
+      <c r="H16" s="25"/>
+    </row>
+    <row r="17" ht="24" customHeight="1" spans="1:9">
+      <c r="A17" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="41" t="s">
+      <c r="B17" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="15" t="s">
+      <c r="C17" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="42" t="s">
-        <v>0</v>
-      </c>
-      <c r="H13" s="42"/>
-      <c r="I13" s="24"/>
-    </row>
-    <row r="14" s="3" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A14" s="12" t="s">
+      <c r="D17" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="E17" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="32"/>
-      <c r="F14" s="15" t="s">
+      <c r="F17" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="G14" s="45" t="s">
+      <c r="G17" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="H14" s="45"/>
-      <c r="I14" s="24"/>
-    </row>
-    <row r="15" s="3" customFormat="1" ht="24" customHeight="1" spans="1:9">
-      <c r="A15" s="27"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="46" t="s">
+      <c r="H17" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="H15" s="46"/>
-      <c r="I15" s="24"/>
-    </row>
-    <row r="16" ht="38" customHeight="1" spans="1:9">
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="47"/>
-      <c r="G16" s="47"/>
-      <c r="H16" s="47"/>
-    </row>
-    <row r="17" ht="24" customHeight="1" spans="1:9">
-      <c r="A17" s="48" t="s">
+    </row>
+    <row r="18" ht="24" customHeight="1" spans="1:9">
+      <c r="A18" s="57"/>
+      <c r="B18" s="57"/>
+      <c r="C18" s="58"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="61"/>
+      <c r="G18" s="60"/>
+      <c r="H18" s="62"/>
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="1:9">
+      <c r="A19" s="57"/>
+      <c r="B19" s="57"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="57"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="57"/>
+      <c r="I19" s="63"/>
+    </row>
+    <row r="20" ht="36" customHeight="1" spans="1:9">
+      <c r="A20" s="64"/>
+      <c r="B20" s="65"/>
+      <c r="C20" s="65"/>
+      <c r="D20" s="65"/>
+      <c r="E20" s="66"/>
+      <c r="F20" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="48" t="s">
+      <c r="G20" s="68"/>
+      <c r="H20" s="69"/>
+      <c r="I20" s="70"/>
+    </row>
+    <row r="21" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="I21" s="71"/>
+    </row>
+    <row r="22" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="A22" s="72"/>
+      <c r="F22" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="49" t="s">
+      <c r="G22" s="74"/>
+      <c r="H22" s="74"/>
+      <c r="I22" s="75"/>
+    </row>
+    <row r="23" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
+      <c r="A23" s="72"/>
+      <c r="F23" s="76" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="50" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="51" t="s">
-        <v>25</v>
-      </c>
-      <c r="F17" s="49" t="s">
-        <v>26</v>
-      </c>
-      <c r="G17" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="H17" s="53" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1" spans="1:9">
-      <c r="A18" s="54"/>
-      <c r="B18" s="54"/>
-      <c r="C18" s="55"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="57"/>
-      <c r="F18" s="58"/>
-      <c r="G18" s="57"/>
-      <c r="H18" s="59"/>
-    </row>
-    <row r="19" ht="24" customHeight="1" spans="1:9">
-      <c r="A19" s="54"/>
-      <c r="B19" s="54"/>
-      <c r="C19" s="49"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="61"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="59"/>
-    </row>
-    <row r="20" ht="24" customHeight="1" spans="1:9">
-      <c r="A20" s="54"/>
-      <c r="B20" s="54"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="57"/>
-      <c r="H20" s="59"/>
-    </row>
-    <row r="21" ht="24" customHeight="1" spans="1:9">
-      <c r="A21" s="54"/>
-      <c r="B21" s="54"/>
-      <c r="C21" s="49"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="61"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="59"/>
-    </row>
-    <row r="22" ht="24" customHeight="1" spans="1:9">
-      <c r="A22" s="54"/>
-      <c r="B22" s="54"/>
-      <c r="C22" s="62"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="61"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="59"/>
-    </row>
-    <row r="23" ht="24" customHeight="1" spans="1:9">
-      <c r="A23" s="63"/>
-      <c r="B23" s="63"/>
-      <c r="C23" s="63"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="63"/>
-      <c r="F23" s="63"/>
-      <c r="G23" s="63"/>
-      <c r="H23" s="63"/>
-      <c r="I23" s="64"/>
-    </row>
-    <row r="24" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A24" s="65"/>
-      <c r="B24" s="66"/>
-      <c r="C24" s="66"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="67"/>
-      <c r="F24" s="68" t="s">
-        <v>29</v>
-      </c>
-      <c r="G24" s="69"/>
-      <c r="H24" s="70"/>
-    </row>
-    <row r="25" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="I25" s="71"/>
-    </row>
-    <row r="26" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A26" s="72"/>
-      <c r="F26" s="73" t="s">
-        <v>30</v>
-      </c>
-      <c r="G26" s="74"/>
-      <c r="H26" s="74"/>
-      <c r="I26" s="26"/>
-    </row>
-    <row r="27" s="4" customFormat="1" ht="15.95" customHeight="1" spans="1:9">
-      <c r="A27" s="72"/>
-      <c r="F27" s="75" t="s">
-        <v>31</v>
-      </c>
-      <c r="G27" s="20"/>
-      <c r="H27" s="76"/>
-      <c r="I27" s="21"/>
-    </row>
-    <row r="28" s="4" customFormat="1" spans="1:9">
-      <c r="I28" s="71"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="77"/>
+      <c r="I23" s="20"/>
+    </row>
+    <row r="24" s="4" customFormat="1" ht="17.6" spans="1:9">
+      <c r="F24" t="s">
+        <v>21</v>
+      </c>
+      <c r="I24" s="71"/>
+    </row>
+    <row r="26" ht="17.6" spans="1:9">
+      <c r="F26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" ht="17.6" spans="1:9">
+      <c r="F27" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I9:I11"/>
   </mergeCells>
   <pageMargins left="0.196850393700787" right="0.236220472440945" top="0.275590551181102" bottom="0.31496062992126" header="0.236220472440945" footer="0.196850393700787"/>
   <pageSetup paperSize="1" scale="80" orientation="portrait" verticalDpi="203"/>
-  <headerFooter alignWithMargins="0" scaleWithDoc="0"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>